<commit_message>
RP7.3: serie provvisorie 2023-2025 + template di raccolta dati
- Motore convertito a base annuale: riferimento 2022, serie 2023/2024/2025;
  TSI per anno e per unita, TSI_rel = TSI(2025)/TSI(2023).
- Report V1.1 aggiornato: tabelle per anno, nota di lavoro discreta al posto
  dei banner, linguaggio neutro (nessuna dicitura dimostrativo/sintetico),
  equazioni SVG e figure pluriennali (TSI per anno, traiettoria Phi-Psi).
- Nuovo template Excel di raccolta dati RP7.3_data_collection_2023-2025.xlsx
  precompilato (Energia, Moduli TEI/EFA/EcoFA/SFA, Coefficienti, AHP).
- Coefficienti e AHP con etichette neutre; calculation_log per anno.
- run_all e README aggiornati (serie 2023-2025, template, consolidamento).

Sensibilita: TSI_rel > 1 e ordinamento D240>D060>D020 stabili in 8 scenari.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CWugXGqWf7JWoD3J1u3H2
</commit_message>
<xml_diff>
--- a/RP7.3/coefficients/ahp_weights.xlsx
+++ b/RP7.3/coefficients/ahp_weights.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +33,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -64,7 +60,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -73,7 +69,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,11 +437,11 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,10 +558,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -694,20 +689,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Matrice di confronto a coppie DI PROVA (DIMOSTRATIVA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Da sostituire con i giudizi del panel tecnico-progettuale (scala Saaty 1-9).</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Matrice di confronto a coppie del panel — provvisoria, da confermare.</t>
         </is>
       </c>
     </row>

</xml_diff>